<commit_message>
chore(data): daily KRZ scrape 2026-04-06
</commit_message>
<xml_diff>
--- a/obwieszczenia_masa_upadlosci.xlsx
+++ b/obwieszczenia_masa_upadlosci.xlsx
@@ -422,14 +422,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
     <col width="56" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -632,32 +632,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20260405/00001</t>
+          <t>20260406/00021</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05.04.2026</t>
+          <t>06.04.2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KR1S/GUp/88/2024</t>
+          <t>SZ1S/GUp-s/64/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Katarzyna</t>
+          <t>Agata</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Jakubowska</t>
+          <t>Cudzanowska</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Skawina, Polska / POLAND</t>
+          <t>Szczecin, Polska / POLAND</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -667,49 +667,39 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>84020202589</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>6751275485</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
-        </is>
-      </c>
+          <t>82070118148</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 5 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza upadłego, którym jest Katarzyna Jakubowska, PESEL 84020202589, sygnatura akt KR1S/GUp/88/2024, na podstawie art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolił syndykowi na sprzedaż z wolnej ręki, po obniżonej cenie, udziału w wysokości 1/2 w prawie własności nieruchomości gruntowej położonej w przy ul. Armii Krajowej 18 w miejscowości Skawina, gm. Skawina, woj. małopolskie, obejmującej działki ewidencyjne nr 5644 i 5645, dla której Sąd Rejonowy w Wieliczce V Zamiejscowy Wydział Ksiąg Wieczystych z s. w Skawinie prowadzi księgę wieczystą nr KR3I/00008006/0 (nr 2.1 w spisie inwentarza), za najwyższą zaoferowaną cenę, nie niższą niż 250.687,50 zł (dwieście pięćdziesiąt tysięcy sześćset osiemdziesiąt siedem złotych 50/100) po przeprowadzeniu przez syndyka pisemnego konkursu ofert, o którym obwieści na co najmniej trzy tygodnie przed terminem rozstrzygnięcia konkursu na co najmniej trzech internetowych portalach branżowych.</t>
+          <t>Syndyk, którym jest Monika Borek, obwieszcza, że dokumentem z dnia 6 kwietnia 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest Agata Cudzanowska (PESEL 82070118148), sygnatura akt SZ1S/GUp-s/64/2026
+obwieszcza:
+w trybie przepisu art. 219 ust. 1d ustawy Prawo upadłościowe, że do akt postępowania upadłościowego Agaty Cudzanowskiej, osoby fizycznej nieprowadzącej działalności gospodarczej, zostały złożone następujące dokumenty: spis inwentarza oraz plan likwidacyjny.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYjRkOWFkY2YtNjVmZC00NjNkLWJhNGItNGNjOWVmOGUxYjMyJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyOTYwNzc1YjMtNzQyZi00YTBlLTkxNWUtYTAwZjI5MzI5YTU3JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20260404/00007</t>
+          <t>20260405/00001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>04.04.2026</t>
+          <t>05.04.2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KR1S/GUp-Sędzia-upr/12/2026</t>
+          <t>KR1S/GUp/88/2024</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -719,12 +709,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Jachyra</t>
+          <t>Jakubowska</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Piotrowice, Polska / POLAND</t>
+          <t>Skawina, Polska / POLAND</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -734,12 +724,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>76032018700</t>
+          <t>84020202589</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5492062327</t>
+          <t>6751275485</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -754,73 +744,140 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie, VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych, ul. Przy Rondzie 7, 31-547 Kraków, obwieszcza, że postanowieniem z 4 kwietnia 2026 roku wydanym przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Katarzyna Jachyra (PESEL 76032018700), sygnatura akt KR1S/GUp-Sędzia-upr/12/2026
-obwieszcza: że w skład masy upadłości nie wchodzi wynagrodzenie upadłej Katarzyny Jachyry w całości, począwszy od miesiąca marca 2026 roku.</t>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 5 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza upadłego, którym jest Katarzyna Jakubowska, PESEL 84020202589, sygnatura akt KR1S/GUp/88/2024, na podstawie art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolił syndykowi na sprzedaż z wolnej ręki, po obniżonej cenie, udziału w wysokości 1/2 w prawie własności nieruchomości gruntowej położonej w przy ul. Armii Krajowej 18 w miejscowości Skawina, gm. Skawina, woj. małopolskie, obejmującej działki ewidencyjne nr 5644 i 5645, dla której Sąd Rejonowy w Wieliczce V Zamiejscowy Wydział Ksiąg Wieczystych z s. w Skawinie prowadzi księgę wieczystą nr KR3I/00008006/0 (nr 2.1 w spisie inwentarza), za najwyższą zaoferowaną cenę, nie niższą niż 250.687,50 zł (dwieście pięćdziesiąt tysięcy sześćset osiemdziesiąt siedem złotych 50/100) po przeprowadzeniu przez syndyka pisemnego konkursu ofert, o którym obwieści na co najmniej trzy tygodnie przed terminem rozstrzygnięcia konkursu na co najmniej trzech internetowych portalach branżowych.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMmJkYzg3ZTgtNjM0ZS00MjE3LWI2ZjUtNzRiNzhhNWNhMDhiJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYjRkOWFkY2YtNjVmZC00NjNkLWJhNGItNGNjOWVmOGUxYjMyJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>20260404/00007</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>04.04.2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>KR1S/GUp-Sędzia-upr/12/2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Katarzyna</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Jachyra</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Piotrowice, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>76032018700</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>5492062327</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie, VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych, ul. Przy Rondzie 7, 31-547 Kraków, obwieszcza, że postanowieniem z 4 kwietnia 2026 roku wydanym przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Katarzyna Jachyra (PESEL 76032018700), sygnatura akt KR1S/GUp-Sędzia-upr/12/2026
+obwieszcza: że w skład masy upadłości nie wchodzi wynagrodzenie upadłej Katarzyny Jachyry w całości, począwszy od miesiąca marca 2026 roku.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMmJkYzg3ZTgtNjM0ZS00MjE3LWI2ZjUtNzRiNzhhNWNhMDhiJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>20260404/00012</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>04.04.2026</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>LU1S/GUp-Sędzia-upr/46/2026</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Łukasz</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Maciąg</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Orchówek, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>77110706933</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>5791764391</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Sąd Rejonowy Lublin-Wschód w Lublinie z siedzibą w Świdniku</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>IX Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 4 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Łukasz Maciąg , PESEL 77110706933, sygnatura akt LU1S/GUp-Sędzia-upr/46/2026, postanowił:
 I.               wyłączyć z masy upadłości Łukasza Maciąga jako osoby fizycznej nieprowadzącej działalności gospodarczej prawa majątkowe w postaci 100 udziałów w spółce LUBAVA SPÓŁKA Z OGRANICZONĄ ODPOWIEDZIALNOŚCIĄ z siedzibą w Warszawie, KRS: 0000620127, o wartości nominalnej 5000 zł (poz. 4.1 spisu inwentarza LU1S/GUp-s/232/2024/154);
@@ -828,65 +885,65 @@
 Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego Lublin-Wschód w Lublinie z siedzibą w Świdniku, IX Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNjY4ODQ3ZjEtNDM1YS00NDQwLTgwNjQtY2FhMWE3NTdiNTRiJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>20260404/00018</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>04.04.2026</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>KR1S/GUp-Sędzia-upr/860/2025</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Małgorzata</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Borkowicz</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Kraków, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>72073114968</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie, VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych, ul. Przy Rondzie 7, 31-547 Kraków, obwieszcza, że postanowieniem z 4 kwietnia 2026 roku wydanym w sprawie upadłościowej osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Małgorzata Borkowicz (PESEL 72073114968), sygnatura akt KR1S/GUp-Sędzia-upr/860/2025
 obwieszcza:
@@ -894,70 +951,70 @@
 II. ustalić, że w skład masy upadłości nie wchodzą środki zgromadzone na rachunku depozytowym Domu Pomocy Społecznej przy ul. Łanowej 1B w Krakowie w kwocie 2 555,27 zł.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyZWU0YWI0ZjItNjhjMi00ZWFlLTk4YjMtYzQxYjcyNDY5ZjE5JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>20260404/00026</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>04.04.2026</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>KR1S/GUp/98/2025</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Edyta</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Pułecka</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Spytkowice, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>76042612080</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 4 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza upadłego, którym jest Edyta Pułecka , PESEL 76042612080, sygnatura akt KR1S/GUp/98/2025, postanowił podstawie art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolić syndykowi na sprzedaż z wolnej ręki, mienia wchodzącego w skład masy upadłości w postaci udziału w wysokości 1/2 części w prawie własności nieruchomości gruntowej zabudowanej, składającej się z działki ewidencyjnej nr 4883/34, o powierzchni 0,0655 ha, położonej w Spytkowicach, woj. małopolskie, objętej księgą wieczystą numer KR1W/00039427/1, za najwyższą zaoferowaną cenę, nie niższą niż wartość oszacowania tj. za kwotę nie niższą niż 318.000,00 zł (trzysta osiemnaście tysięcy złotych 00/100), po przeprowadzeniu przez syndyka pisemnego konkursu ofert, o którym obwieści na co najmniej dwa tygodnie przed terminem rozstrzygnięcia konkursu w prasie o zasięgu lokalnym oraz na co najmniej dwóch internetowych portalach branżowych.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYjU3MWM5NzItYzE3Ni00Yzc2LTliNWItODJkZDFhMzBiMmYzJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
@@ -972,6 +1029,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(data): daily KRZ scrape 2026-04-07
</commit_message>
<xml_diff>
--- a/obwieszczenia_masa_upadlosci.xlsx
+++ b/obwieszczenia_masa_upadlosci.xlsx
@@ -422,15 +422,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="56" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -510,32 +510,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20260406/00017</t>
+          <t>20260407/00001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06.04.2026</t>
+          <t>07.04.2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SZ1S/GUp-s/61/2026</t>
+          <t>BI1B/GUp-Sędzia-upr/44/2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Zbigniew</t>
+          <t>EWELINA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Banach</t>
+          <t>PODGÓRSKA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Uniemyśl, Polska / POLAND</t>
+          <t>Zbroszki, Polska / POLAND</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -545,58 +545,62 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>54032407177</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>8512599352</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+          <t>94030412982</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Białymstoku</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>VIII Wydział Gospodarczy</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Syndyk, którym jest Monika Borek, obwieszcza, że dokumentem z dnia 6 kwietnia 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest Zbigniew Banach (PESEL 54032407177), sygnatura akt SZ1S/GUp-s/61/2026
+          <t>Sąd Rejonowy w Białymstoku, VIII Wydział Gospodarczy, ul. Adama Mickiewicza 103, 15-950 Białystok, obwieszcza, że dokumentem z dnia7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest EWELINA PODGÓRSKA (PESEL 94030412982), sygnatura akt BI1B/GUp-Sędzia-upr/44/2026
 obwieszcza:
-w trybie przepisu art. 219 ust. 1d ustawy Prawo upadłościowe, że do akt postępowania upadłościowego Zbigniewa Banacha, osoby fizycznej nieprowadzącej działalności gospodarczej, zostały złożone następujące dokumenty: spis inwentarza oraz plan likwidacyjny.</t>
+1. wyłączyć z masy upadłości samochód osobowy Ford Fiesta 1.4 o numerze rejestracyjnym WPU 53694, rok produkcji 2010</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNzFjOWJmN2YtOTE1MS00YjRhLTg2NDYtYmY2ZWRlNTA4YWE3JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNzk4ZjU4M2QtMzRjYi00MDQwLTlhZjAtZTFjNDgxMWFkYWM5JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>20260406/00019</t>
+          <t>20260407/00063</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06.04.2026</t>
+          <t>07.04.2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SZ1S/GUp-s/61/2026</t>
+          <t>KR1S/GUp/70/2023</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Zbigniew</t>
+          <t>Wioletta</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Banach</t>
+          <t>Urbańska-Staszkiewicz</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Uniemyśl, Polska / POLAND</t>
+          <t>Kraków, Polska / POLAND</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -606,58 +610,68 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>54032407177</t>
+          <t>87102204208</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>8512599352</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+          <t>6751317410</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Syndyk, którym jest Monika Borek, obwieszcza, że dokumentem z dnia 6 kwietnia 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest Zbigniew Banach (PESEL 54032407177), sygnatura akt SZ1S/GUp-s/61/2026
-obwieszcza:
-w trybie przepisu art. 219 ust. 1d ustawy Prawo upadłościowe, że do akt postępowania upadłościowego Zbigniewa Banacha osoby fizycznej nieprowadzącej działalności gospodarczej, został złożony następujący dokument: korekta planu likwidacyjnego.</t>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 25 lutego 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza dłużnika, którym jest Wioletta Urbańska-Staszkiewicz, PESEL 87102204208, prowadzonej pod sygn. akt KR1S/GUp/70/2023, postanowił:
+I. wyłączyć z masy upadłości:
+1) udział spadkowy w wysokości 1/4 w spadku po ojcu upadłej - Kazimierzu Urbańskim, stanowiący ogół praw i obowiązków majątkowych, z wyłączeniem lokalu mieszkalnego objętego księgą wieczystą KR1P/00385735/8 (poz. 4.1 w spisie inwentarza),
+2) udział spadkowy w wysokości 1/2 w spadku po bracie upadłej - Jacku Urbańskim, stanowiący ogół praw i obowiązków majątkowych, z wyłączeniem lokalu mieszkalnego objętego księgą wieczystą KR1P/00385735/8 (poz. 4.2 w spisie inwentarza);
+II. na podstawie art. 357 § 6 k.p.c. w zw. z art. 229 ust. 1 prawa upadłościowego odstąpić od uzasadnienia niniejszego postanowienia wobec uznania w całości zasadności żądania wniosku syndyka i przytoczonych na jego poparcie argumentów przedstawionych szczegółowo w piśmie syndyka z dnia 16 stycznia 2026 roku.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyOTNlMWYzOTUtMDQ5Ny00MGNjLTliNDUtMzRjNTRiNDllMTkxJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMjE4NmQ5YzItZDM1Ny00OGFiLTgwYmQtMmE0MzRjNGQ4ZTZjJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>20260406/00021</t>
+          <t>20260407/00067</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06.04.2026</t>
+          <t>07.04.2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SZ1S/GUp-s/64/2026</t>
+          <t>BY1B/GUp-s/107/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Agata</t>
+          <t>NATALIA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Cudzanowska</t>
+          <t>MOTYKA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Szczecin, Polska / POLAND</t>
+          <t>Markowice, Polska / POLAND</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -667,7 +681,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>82070118148</t>
+          <t>91070515565</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -675,209 +689,2179 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
+          <t>Syndyk masy upadłości w sprawie upadłościowej Natalii Motyki nieprowadzącej działalności gospodarczej w upadłości, sygn. akt: BY1B/GUp-s/107/2026, na podstawie art. 491¹¹a prawa upadłościowego, zawiadamia o wyborze sposobu likwidacji składnika masy upadłości w postaci prawa własności lokalu mieszkalnego nr 18, położonego w Markowicach 43 a o pow. 29,56 m2 dla którego Sąd Rejonowy w Mogilnie prowadzi KW nr BY1M/00020182/3 oraz udziału 1/12 w prawie własności nieruchomości zabudowanej położonej w Markowicach, gmina Strzelno, dz. nr 126/7 o pow.415 m2 objętej KW nr BY1M/00019208/2.
+1.     Syndyk sporządził spis inwentarza oraz przyjął wartość prawa własności lokalu mieszkalnego nr 18, położonego w Markowicach 43 a o pow. 29,56 m2 dla którego Sąd Rejonowy w Mogilnie prowadzi KW nr BY1M/00020182/3, zgodnie z operatem szacunkowym sporządzonym przez rzeczoznawcę majątkowego Pawła Michalskiego w kwocie 107.000,00 zł oraz udziału 1/12 w prawie własności nieruchomości zabudowanej położonej w Markowicach, gmina Strzelno, dz. nr 126/7 o pow.415 m2 objętej KW nr BY1M/00019208/2, zgodnie z operatem szacunkowym sporządzonym przez rzeczoznawcę majątkowego Pawła Michalskiego w kwocie 4.667,00 zł.
+2.     W przypadku braku wstrzymania likwidacji przez Sąd, syndyk przystąpi do sprzedaży powyższego majątku z wolnej ręki poprzez umieszczenie ogłoszenia o sprzedaży za cenę nie niższą niż 111.667,00 zł na portalu internetowym OLX.
+3.     W przypadku braku wpływu ofert zakupu w wyznaczonym do tego terminie za powyższą kwotę, syndyk będzie obniżał cenę sprzedaży nieruchomości o kolejne 10 % ceny wyszacowania, po upływie każdego terminu do składania ofert, aż do momentu pozyskania nabywcy.
+Pouczenia:
+Art. 49111a. [Wybór sposobu likwidacji masy upadłości]
+1.   Wyboru sposobu likwidacji masy upadłości dokonuje samodzielnie syndyk w sposób, który umożliwia zaspokojenie wierzycieli w jak największym stopniu, z uwzględnieniem kosztów likwidacji.
+2.   O wyborze sposobu likwidacji nieruchomości oraz wyborze sposobu likwidacji składników masy upadłości, których wartość oszacowania wskazana w spisie inwentarza przekracza pięciokrotność przeciętnego miesięcznego wynagrodzenia w sektorze przedsiębiorstw bez wypłat nagród z zysku w trzecim kwartale roku poprzedzającego złożenie spisu inwentarza, ogłoszonego przez Prezesa Głównego Urzędu Statystycznego, syndyk zawiadamia wierzycieli oraz sąd za pośrednictwem systemu teleinformatycznego obsługującego postępowanie sądowe z wykorzystaniem udostępnianych w tym systemie formularzy. W zawiadomieniu syndyk wskazuje sposób likwidacji oraz minimalną cenę.
+3.   Na skutek skargi na czynności syndyka, o której mowa w art. 49112a, lub z urzędu sąd, w drodze postanowienia, zakazuje syndykowi dokonania likwidacji składnika masy upadłości w wybrany przez syndyka sposób lub za wskazaną minimalną cenę, jeżeli likwidacja byłaby niezgodna z prawem albo prowadziłaby do pokrzywdzenia upadłego lub wierzycieli.
+4.   Przed wydaniem postanowienia, o którym mowa w ust. 3, sąd może wstrzymać dokonanie likwidacji składnika masy upadłości. O wstrzymaniu likwidacji składnika masy upadłości sąd zawiadamia syndyka w dniu wydania postanowienia o wstrzymaniu likwidacji.
+5.   W przypadku braku wstrzymania lub zakazu likwidacji składnika masy upadłości likwidacja może nastąpić po upływie czternastu dni od dnia zawiadomienia, o którym mowa w ust. 2.
+Art. 49112a. [Skarga na czynności syndyka]
+1.   Na czynności syndyka przysługuje skarga do sądu upadłościowego. Dotyczy to także zaniechania przez syndyka dokonania czynności.
+2.   Skargę może złożyć upadły, wierzyciel lub inna osoba, której prawo zostało przez czynności lub zaniechanie syndyka naruszone albo zagrożone.
+3.   Skarga powinna czynić zadość wymaganiom pisma procesowego oraz określać zaskarżoną czynność lub czynność, której zaniechano, jak również wniosek o zmianę, uchylenie lub dokonanie czynności, wraz z uzasadnieniem.
+4.   Skargę wnosi się w terminie siedmiu dni od dnia dokonania czynności, gdy upadły, wierzyciel lub osoba, której prawo zostało przez czynność syndyka naruszone albo zagrożone, była przy czynności obecna lub była o jej terminie zawiadomiona; w innych przypadkach - od dnia zawiadomienia o dokonaniu czynności upadłego, wierzyciela lub osoby, której prawo zostało przez czynność syndyka naruszone albo zagrożone, a w braku zawiadomienia - od dnia powzięcia wiadomości przez skarżącego o dokonanej czynności. Skargę na zaniechanie przez syndyka dokonania czynności wnosi się w terminie siedmiu dni od dnia, w którym skarżący dowiedział się, że czynność miała być dokonana.
+5.   Skargę wnosi się do syndyka, który dokonał zaskarżonej czynności lub zaniechał jej dokonania. Syndyk w terminie trzech dni od dnia otrzymania skargi sporządza uzasadnienie zaskarżonej czynności, o ile nie zostało ono sporządzone wcześniej, albo przyczyn jej zaniechania i przekazuje je wraz ze skargą do właściwego sądu upadłościowego, chyba że skargę w całości uwzględnia. O uwzględnieniu skargi syndyk zawiadamia skarżącego oraz zainteresowanych, których uwzględnienie skargi dotyczy, za pośrednictwem systemu teleinformatycznego obsługującego postępowanie sądowe z wykorzystaniem udostępnianych w tym systemie formularzy.
+6.   Sąd rozpoznaje skargę w terminie siedmiu dni od dnia jej wpływu do sądu, a gdy skarga zawiera braki formalne, które podlegają uzupełnieniu - od dnia jej uzupełnienia.
+7.   Wniesienie skargi nie wstrzymuje postępowania upadłościowego ani dokonania zaskarżonej czynności, chyba że sąd wstrzyma dokonanie czynności.
+8.   Sąd odrzuca skargę wniesioną po upływie przepisanego terminu, nieopłaconą lub z innych przyczyn niedopuszczalną, jak również skargę, której braków nie uzupełniono w terminie. Na postanowienie sądu o odrzuceniu skargi służy zażalenie.
+9.   W razie odrzucenia skargi sąd z urzędu bierze pod uwagę okoliczności wskazane w skardze i w razie potrzeby wydaje syndykowi polecenie dokonania odpowiednich czynności lub zakazuje syndykowi dokonania określonych czynności.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNGM0NjA4YmQtMmZmOS00YTFiLWJiMDgtNDFhMmYwMTI4MGQ4JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>20260407/00073</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>WA2M/GUp-s/374/2024</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Anna</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Szkodzińska</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Warszawa, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>00221409523</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>sygn. akt WA2M/GUp-s/374/2024, znak pisma: WA2M/GUp-s/374/2024/167
+Treść obwieszczenia syndyka
+Dnia 3 kwietnia 2026 roku
+Syndyk obwieszcza, że w postępowaniu upadłościowym dłużnika, którym jest Anna Szkodzińska, prowadzonego pod sygn. akt: WA2M/GUp-s/374/2024, złożono do akt opis i szacowanie:
+nieruchomości: udział 3/8 w prawie własności nieruchomości gruntowej, stanowiącej dz. ew. nr 301 położonej w miejscowości Nuna, gm. Nasielsk, pow. nowodworski, woj. mazowieckie. Dla nieruchomości prowadzona jest księga wieczysta nr OS1U/00037691/4 przez Sąd Rejonowy w Pułtusku, IV Wydział Ksiąg Wieczystych.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNzc1YzliYjQtY2QxNi00ZDY2LTgyMTktOWZmNGEwMjk3MzRhJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>20260407/00099</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GD1G/GUp/90/2023</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>8421775116</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy Gdańsk-Północ w Gdańsku</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>VI Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 3 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości upadłego, którym jest HIMET SPÓŁKA Z OGRANICZONĄ ODPOWIEDZIALNOŚCIĄ SPÓŁKA KOMANDYTOWA, KRS 0000659576, sygnatura akt GD1G/GUp/90/2023, postanowił:
+I. na podstawie art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolić syndykowi na sprzedaż z wolnej ręki mienia wchodzącego w skład masy upadłości upadłego HIMET SPÓŁKA Z OGRANICZONĄ ODPOWIEDZIALNOŚCIĄ SPÓŁKA KOMANDYTOWA w postaci:
+wielkogabarytowe 5 osiowe Centrum obróbcze C9-Ciman Mira (nr inw. 1.1), za cenę nie niższą niż kwota 55.370,00 zł netto;
+wielkogabarytowe 4 osiowe centrum obróbcze CHIRON FZ 18 (nr inw. 1.2), za cenę nie niższą niż kwota 6.979,00 zł netto;
+6 kompletów elementów do maszyn HIMLET MAGNETIK stanowiące części stalowe (nr inw. 1.3), za cenę nie niższą niż kwota 100.905,00 zł netto;
+piła taśmowa Pilous (nr inw. 1.5), za cenę nie niższą niż kwota 5.320,00 zł netto;
+maszyna w budowie dla firmy Flader FM Palczewski MIKUS s.c. (nr inw. 1.6) składająca się z: część elektrowrzeciono HITEKO NOWE, wiertarka wielowrzecionowa nowa, obrabiarka pięcioosiowa CNC - nieskończona oraz szafa z elektroniką, za cenę nie niższą niż kwota 166.250,00 zł netto.
+II. wniosek Syndyka z dn. 30 marca 2026 roku (nr dokumentu: GD1G/GUp/90/2023/78) uczynić integralną częścią niniejszego postanowienia.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMjY4ZmYzNTAtZjIwNi00YzMwLWI0Y2ItMmZkOTA5ZjcwN2ZhJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>20260407/00105</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>WA2M/GUp-s/219/2025</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dariusz</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pańczyk</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Warszawa, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>71082113535</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>sygn. akt WA2M/GUp-s/219/2025, znak pisma: WA2M/GUp-s/219/2025/51
+Treść obwieszczenia syndyka
+Dnia 3 kwietnia 2026 roku
+Syndyk obwieszcza, że w postępowaniu upadłościowym dłużnika, którym jest Dariusz Pańczyk, prowadzonego pod sygn. akt: WA2M/GUp-s/219/2025, złożono do akt opis i szacowanie:
+nieruchomości: udział 1/2 w prawie własności nieruchomości gruntowej niezabudowanej stanowiącej dz. ew. nr 95/11, obręb 0013, położonej przy ul. Działkowej 20, na terenie miejscowości Warzenko, gmina Przodkowo, powiat kartuski, woj. pomorskiego. Dla nieruchomości prowadzona jest księga wieczysta nr GD1R/00053765/9 przez Sąd Rejonowy w Kartuzach, V Wydział Ksiąg Wieczystych.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMjJiZGRjNTEtZDdkMS00MzFmLTgxNTUtMGMxMDBhZWRiZWZjJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>20260407/00106</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ZG1E/GUp-Sędzia-upr/24/2026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Paulina</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Urbanowicz-Mróz</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Zielona Góra, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>88093005320</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Zielonej Górze</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>V Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Zielonej Górze, V Wydział Gospodarczy, pl. Słowiański 12, 65-069 Zielona Góra, obwieszcza, że postanowieniem sędziego wyznaczonego z dnia 3 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Paulina Urbanowicz-Mróz (PESEL 88093005320), sygnatura akt ZG1E/GUp-Sędzia-upr/24/2026
+postanowiono:
+na podstawie art. 63 ust. 1c Prawa upadłościowego określić część dochodu upadłej, która nie wchodzi do masy upadłości, w zakresie obejmującym środki pieniężne uzyskane z tytułu zwrotu podatku dochodowego od osób fizycznych upadłej za 2025 r.;
+na podstawie art. 357 § 6 k.p.c. w zw. z art. 229 ust. 1 Prawa upadłościowego uwzględnić w całości wniosek upadłej oraz podzielić zawarte w nim argumenty i odstąpić od uzasadnienia postanowienia, o którym mowa w pkt 1.
+Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego w Zielonej Górze, V Wydział Gospodarczy. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMGQ4YzFiMmEtNzY3Ny00NjFmLWJmMGItY2Q5ZDNlOWNmMDYzJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20260407/00107</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PO1P/GUp-Sędzia-upr/1502/2025</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Marcin</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Wdowczyk</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Poznań, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>83061818753</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>6181937126</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy Poznań-Stare Miasto w Poznaniu</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>XI Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy Poznań-Stare Miasto w Poznaniu, XI Wydział Gospodarczy, ul. Młyńska 1a, 61-729 Poznań, obwieszcza, że dokumentem z dnia 29 stycznia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Marcin Wdowczyk (PESEL 83061818753), sygnatura akt PO1P/GUp-Sędzia-upr/1502/2025
+obwieszcza: oddalić wniosek pełnomocnika upadłego o wyłączenie z masy upadłości udziałów przysługujących upadłemu w następujących spółkach:
+MARWIPOL spółka z ograniczoną odpowiedzialnością, KRS: 0001149696;
+SUNPOWERTECH spółka z ograniczoną odpowiedzialnością, KRS: 0000595478;
+FORTENZA spółka z ograniczoną odpowiedzialnością, KRS: 0001193113.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMDA4MmU0MjEtOTQzZi00MTMxLWJmMjQtMTI0ZjQ4NDE1YzQzJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>20260407/00150</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BB1B/GUp-Sędzia-upr/149/2026</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Ewa</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Szczygieł</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Bielsko-Biała, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>55070119686</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Bielsku-Białej</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>VI Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Ewa Szczygieł, PESEL 55070119686, prowadzonej pod sygn. akt BB1B/GUp-Sędzia-upr/149/2026,
+postanowił:
+wyłączyć z masy upadłości całość świadczenia emerytalnego, które obecnie wynosi 3 335,23zł,
+odstąpić od sporządzenia uzasadnienia pkt 1 postanowienia (wniosek upadłego z dnia 1.04.2026r. oraz pismo syndyka z dnia 1.04.2026r.).
+Poucza się, że wierzycielowi przysługuje zażalenie na postanowienie o wyłączeniu z masy upadłości. Zażalenie wnosi się w następujący sposób: wierzyciel może w terminie tygodnia od dnia obwieszczenia postanowienia o wyłączeniu z masy upadłości, wnieść zażalenie. Zażalenie podlega opłacie w wysokości 200,00 zł. Sąd odrzuci zażalenie jeżeli będzie ono spóźnione, nieopłacone lub dotknięte brakami, które nie zostaną usunięte mimo wezwania. Zażalenie należy skierować do Sądu Upadłościowego - Sądu Rejonowego w Bielsku-Białej, VI Wydział Gospodarczy.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMmI3NjU3MmMtNjc2Ni00NGVjLWEwMzYtN2UwMGZjNTMyMzU5JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>20260407/00173</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KA1K/GUp/16/2023</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Zbigniew</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Nędza</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Czeladź, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>52060202575</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>6251439222</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy Katowice Wschód w Katowicach</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>X Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Syndyk masy upadłości w postępowaniu upadłościowym osoby fizycznej nieprowadzącej działalności gospodarczej Zbigniewa Nędzy PESEL 52060202575, NIP 6251439222 sygn. akt: KA1K/GUp/16/2023, zawiadamia o sporządzeniu opisu i oszacowania przysługującego upadłemu udziału 1/2 w nieruchomości gruntowej zabudowanej w skład której wchodzą działki ewidencyjne nr 5312/227, 5312/341, 5312/478, tworzące całość funkcjonalną o łącznej powierzchni 1104 m2, położonej przy ul. Czarne 13 w Wiśle, dla której Sąd Rejonowy w Cieszynie, V Wydział Ksiąg Wieczystych prowadzi księgę wieczystą o numerze BB1C/00089309/1.
+Z treścią opisu i oszacowania uczestnicy postępowania i osoby zainteresowane mogą zapoznać się po uzyskaniu dostępu do akt postępowania w systemie Krajowego Rejestru Zadłużonych. W terminie tygodnia od daty ukazania się niniejszego obwieszczenia można wnieść do sędziego wyznaczonego zarzuty przeciwko opisowi i oszacowaniu. W postępowaniu upadłościowym pisma procesowe oraz dokumenty, z wyłączeniem pism i dokumentów, o których mowa w art. 216ab, wnosi się wyłącznie za pośrednictwem systemu teleinformatycznego obsługującego postępowanie sądowe z wykorzystaniem udostępnianych w tym systemie formularzy. Pisma oraz dokumenty niewniesione za pośrednictwem systemu teleinformatycznego obsługującego postępowanie sądowe nie wywołują skutków prawnych, jakie ustawa wiąże z wniesieniem pisma albo dokumentu do sądu, tymczasowego nadzorcy sądowego, zarządcy przymusowego, syndyka albo organu, do którego przepisy o syndyku stosuje się odpowiednio.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNTk5MTg1OWMtYjNjNC00MWRiLTg2MWMtYzhkMGIwZGVmMTMxJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>20260407/00189</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KI1L/GUp/99/2025</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mariusz</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Pietrala</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Kielce, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>68072911392</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>6571000812</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Kielcach</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>V Wydział Gospodarczy Sekcja ds. Upadłościowych i Restrukturyzacyjnych</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz w postępowaniu po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza prowadzonym wobec dłużnika, którym jest Mariusz Pietrala (PESEL 68072911392), sygnatura akt KI1L/GUp/99/2025, zarządził:
+o obwieszczeniu, iż syndyk sporządził i przekazał sędziemu-komisarzowi w dniu 3 kwietnia 2026 r. opis i oszacowanie nieruchomości gruntowej położonej w Kielcach przy ul. Skrajnej (dz.ew. nr 504) dla której Sąd Rejonowy w Kielcach VI Wydział Ksiąg Wieczystych prowadzi księgę wieczystą nr KI1L/00051887/0. 
+Zarzuty na opis i oszacowanie wnosi się w terminie tygodnia od dnia obwieszczenia o ich przekazaniu sędziemu-komisarzowi. Zarzuty rozpoznaje sędzia-komisarz.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNzYwY2JhNGMtOGNlYy00M2RkLTllN2MtNTY4MWMwZDQxY2EwJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20260407/00210</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TR1T/GUp-Sędzia-upr/14/2026</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Zygmunt</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sokołowski</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Tarnów, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>58041319052</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>8731168876</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Tarnowie</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>V Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Sędzia wyznaczony obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Zygmunt Sokołowski, PESEL 58041319052, sygnatura akt TR1T/GUp-Sędzia-upr/14/2026, postanowił:
+wyłączyć z masy upadłości dłużnika Zygmunta Sokołowskiego składniki majątkowe w postaci:
+a. 50 (pięćdziesięciu) udziałów w Jazymi spółce z ograniczoną odpowiedzialnością w Krakowie (KRS: 0000503509), oznaczonych w spisie inwentarza numerem 4.1. o wartości nominalnej 2.500 zł (dwa tysiące pięćset złotych);
+b. 50 (pięćdziesięciu) udziałów w Comet Enterprise spółce z ograniczoną odpowiedzialnością w Krakowie (KRS: 0000512359), oznaczonych w spisie inwentarza numerem 4.2. o wartości nominalnej 2.500 zł (dwa tysiące pięćset złotych).
+Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego w Tarnowie, V Wydział Gospodarczy. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyOTY5YWYxODMtOWUwOS00YjZkLTk3MmUtZTM2Zjk3ODVhYjJkJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>20260407/00235</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LU1S/GUp-s/28/2026</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Stawiński</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Matczyn, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>83122403151</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>7132763879</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>sygn. akt LU1S/GUp-s/28/2026, znak pisma: LU1S/GUp-s/28/2026/41
+Treść obwieszczenia syndyka
+Dnia 6 kwietnia 2026 roku
+Syndyk obwieszcza, że w postępowaniu upadłościowym dłużnika, którym jest Adam Stawiński, prowadzonego pod sygn. akt: LU1S/GUp-s/28/2026, złożono do akt opis i szacowanie:
+nieruchomości gruntowej objętej księgą wieczystą nr KR1I/00047965/1, stanowiąca działki ewid. nr 1584/9 i 1587/5 o łącznej powierzchni 705 m2, zabudowanej budynkiem mieszkalnym jednorodzinnym nr 1084 zrealizowanym w zabudowie wolnostojącej, położonej w Węgrzcach Wielkich, jednostce ewid. Wieliczka - G, obrębie ewid. nr 28, Węgrzce Wielkie, wraz z udziałem w nieruchomości gruntowej ujętej w księdze wieczystej nr KR1I/00045203/8, odpowiadającej działkom ewid. nr 1587/11, 1589/9, 1586/6, 1588/19, 1588/9, stanowiącej drogę wewnętrzną.
+Na opis i oszacowanie można wnosić zarzuty w terminie tygodnia od dnia niniejszego obwieszczenia. Zarzuty wnosi się do sędziego-wyznaczonego na adres: Sąd Rejonowy Lublin –Wschód w Lublinie z siedzibą w Świdniku, IX Wydział Gospodarczy ds. Upadłościowych i Restrukturyzacyjnych, ul. Kardynała Stefana Wyszyńskiego 18, 21-040 Świdnik.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNTczMmQ1NWEtOThiMi00MzA0LWJjYjgtYTlhZmFhMzUyNWIxJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>20260407/00258</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SW1W/GUp-Sędzia-upr/55/2026</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mateusz</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Szulc</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Dzierżoniów, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>90050916275</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>6423134857</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Wałbrzychu</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>VI Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Mateusz Szulc, PESEL 90050916275, sygnatura akt SW1W/GUp-Sędzia-upr/55/2026, postanowił:
+wyłączyć z masy upadłości: Ford Transit, nr rejestracyjny PZ 0241Y, rok produkcji 2007, nr VIN WF0XXXTTFX7J73858 .
+Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego w Wałbrzychu, VI Wydział Gospodarczy. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyZDBlNjJlMDAtYzlkYy00OTAzLWI4NTctYWNjYmVlN2M0NDUyJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>20260407/00269</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SW1W/GUp-Sędzia-upr/138/2026</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Piotr</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Skowera</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Wałbrzych, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>83042309135</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>8862589584</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Wałbrzychu</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>VI Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Wałbrzychu, VI Wydział Gospodarczy, ul. Juliusza Słowackiego 10,11,11a, 58-300 Wałbrzych, obwieszcza, że dokumentem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Piotr Skowera (PESEL 83042309135), sygnatura akt SW1W/GUp-Sędzia-upr/138/2026
+obwieszcza:
+wyłączyć z masy upadłości Piotra Skowery samochód osobowy marki Ford Focus, rok produkcji 2012, nr rejestracyjny DBA32415.
+Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego w Wałbrzychu, VI Wydział Gospodarczy. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMWIzNTk3MzAtYTNhYi00MTY0LWExNjQtZGUxNjI1NjRmNmE2JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20260407/00299</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BY1B/GUp/18/2022</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TOMASZ</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GÓRALSKI</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Inowrocław, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>56102807155</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>5561014019</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Bydgoszczy</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>XV Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza upadłego, którym jest TOMASZ GÓRALSKI, PESEL 56102807155, sygnatura akt BY1B/GUp/18/2022, postanowił: na podstawie art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolić syndykowi na sprzedaż z wolnej ręki mienia w postaci udziału wynoszącego 1/2 w prawie własności nieruchomości zabudowanej położonej w miejscowości Marcinkowo, gm. Inowrocław:
+a) stanowiącej działkę nr 58/6, dla której Sąd Rejonowy w Inowrocławiu prowadzi księgę wieczystą KW nr BY1I/00027957/2, za cenę nie niższą niż 40% wartości oszacowania, tj. 232 400 (dwieście trzydzieści dwa tysiące czterysta) złotych,
+b) stanowiącej działkę nr 58/5, dla której Sąd Rejonowy w Inowrocławiu prowadzi księgę wieczystą KW nr BY1I/00057356/8, za cenę nie niższą niż 40% wartości oszacowania, tj. 109 400 (sto dziewięć tysięcy czterysta) złotych,
+c) stanowiącej działkę nr 58/7, dla której Sąd Rejonowy w Inowrocławiu prowadzi księgę wieczystą KW nr BY1I/00057357/5, za cenę nie niższą niż 40% wartości oszacowania, tj. 207 600 (dwieście siedem tysięcy sześćset) złotych,
+d) stanowiącej działkę nr 58/8, dla której Sąd Rejonowy w Inowrocławiu prowadzi księgę wieczystą KW nr BY1I/00057358/2, za cenę nie niższą niż 40% wartości oszacowania, tj. 149 200 (sto czterdzieści dziewięć tysięcy dwieście) złotych.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNWY0ZTgzMWEtNjIxNy00ZjhiLWE3MTMtNjBkN2IwNzlhNGFhJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>20260407/00337</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OL1O/GUp-Sędzia-upr/143/2026</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Jacek</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Czechowski</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Szczytno, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>53091201573</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>7450002600</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Olsztynie</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>V Wydział Gospodarczy Sekcja ds. Upadłościowych i Restrukturyzacyjnych</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Jacek Czechowski, PESEL 53091201573, sygnatura akt OL1O/GUp-Sędzia-upr/143/2026, postanowił:
+wyłączyć z masy upadłości udziały członkowskie upadłego w Banku Spółdzielczym w Szczytnie w wysokości 200 zł.
+Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego w Olsztynie, V Wydział Gospodarczy Sekcja ds. Upadłościowych i Restrukturyzacyjnych. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMzdjNWI0NDUtMmYzNC00ZWU1LWFmOWQtYjhmODhiYjllOTFhJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>20260407/00397</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>KI1L/GUp/29/2024</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Sławomir</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Michalec</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Kielce, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>63042609855</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>9590217508</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Kielcach</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>V Wydział Gospodarczy Sekcja ds. Upadłościowych i Restrukturyzacyjnych</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz w postępowaniu po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza prowadzonym wobec dłużnika, którym jest Sławomir Michalec (PESEL 63042609855), sygnatura akt KI1L/GUp/29/2024, zarządził:
+o obwieszczeniu, iż syndyk sporządził i przekazał sędziemu-komisarzowi w dniu 2 kwietnia 2026 r. opis i oszacowanie udziału wynoszącego 1/2 w prawie współwłasności nieruchomości lokalowej nr 11, przy ul. Karbońskiej 4 w Kielcach.
+Zarzuty na opis i oszacowanie wnosi się w terminie tygodnia od dnia obwieszczenia o ich przekazaniu sędziemu-komisarzowi. Zarzuty rozpoznaje sędzia-komisarz.</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNTY4M2NiMGQtZGVjYi00NWFjLWIzYmEtNDg0OWY4NmYyMTMzJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20260407/00400</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OP1O/GUp-Sędzia-upr/21/2026</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>OLGA</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>KUBICA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Dytmarów, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>87062316609</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Opolu</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>V Wydział Gospodarczy Sekcja ds. Upadłościowych i Restrukturyzacyjnych</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Sędzia wyznaczony obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest OLGA KUBICA, PESEL 87062316609, prowadzonej pod sygn. akt OP1O/GUp-Sędzia-upr/21/2026, postanowił:
+na podstawie art. 63 ust. 1 pkt 1 w zw. z art. 4912 ust. 1 ustawy z dnia 28 lutego 2003 r. Prawo upadłościowe w zw. z art. 829 pkt 6 k.p.c. stwierdzić, że samochód osobowy marki Volkswagen Turan, numer rejestracyjny OPR6F7, rok produkcji 2010, ujawniony w spisie inwentarza pod numerem 1.1 nie wchodzi w skład masy upadłości.
+Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego w Opolu, V Wydział Gospodarczy Sekcja ds. Upadłościowych i Restrukturyzacyjnych. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYWIwZGIzZDAtZDQwYS00MWVkLTkzMGMtYzA1MzE3YTExNTJlJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20260407/00425</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ZG1E/GUp-s/2/2026</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Tomasz</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Szymański</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Czerwieńsk, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>76010604019</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>9730245078</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Informuje się, że w postępowaniu upadłościowym upadłego, którym jest Tomasz Szymański PESEL 76010604019, prowadzonego pod sygn. akt: ZG1E/GUp-s/2/2026 złożono do akt opis i oszacowanie prawa własności nieruchomości gruntowej niezabudowanej, położonej w Nietkowie, gmina Czerwieńsk, województwo lubuskie, oznaczonej jako działka nr 963/2, dla której prowadzona jest księga wieczysta ZG1E/00099879/8 oraz prawa własności nieruchomości gruntowej niezabudowanej, położonej w Nietkowie, gmina Czerwieńsk, województwo lubuskie, oznaczonej jako działka nr 347/5, dla której prowadzona jest księga wieczysta ZG1E/00008006/4.
+Poucza się, że na opis i oszacowanie można wnieść zarzuty. Zarzuty wnosi się w terminie tygodnia od dnia ukazania się niniejszego obwieszczenia sędziemu-komisarzowi albo w przypadku postępowania upadłościowego prowadzonego na podstawie art. 491 (1) ust. 1 prawa upadłościowego sędziemu wyznaczonemu.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNmY2NGQ3MDctY2E3ZS00YjI4LWJjNDUtYjhmNGQxOTcyYjYxJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>20260407/00440</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>WA2M/GUp/1/2025</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Jabłoński</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Warszawa, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>85021600116</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>7010012994</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy dla m.st.Warszawy w Warszawie</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>XIX Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza upadłego, którym jest Daniel Jabłoński, PESEL 85021600116, sygnatura akt WA2M/GUp/1/2025, postanowił:
+na podstawie art. 4911 ust. 2 w zw. art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolić syndykowi na sprzedaż z wolnej ręki mienia wchodzącego w skład masy upadłości upadłego, którym jest Daniel Jabłoński, w postaci należności od Lazzoni Group sp. z o.o. sp.k. (składnik masy upadłości w spisie inwentarza numer 5.1 oraz w uzupełniającym spisie inwentarza nr 5.3) przysługującej solidarnie również Rafałowi Grucy, wobec którego toczy się postępowania upadłościowe pod sygnaturą WA2M/GUp/2/2025, o wartości nominalnej 85.000 zł za 50% ceny wynikającej z oszacowania (wartość rynkowa na podstawie Oszacowania z dnia 20 marca 2026 r. sporządzonego przez biegłego sądowego Wojciecha Makucia, dołączonej do akt postępowania upadłościowego pod nr 147, znak w aktach WA2M/GUp/2/2025/147) , czyli:
+1.   za cenę nie niższą niż 3.128,00 zł (słownie: trzy tysiące sto dwadzieścia osiem złotych) netto, przy czym syndyk przeprowadzi aukcję podaną do publicznej wiadomości, w terminie nie wcześniejszym niż po upływie dwóch tygodni od dnia wydania przez Sędziego-Komisarza niniejszego postanowienia;
+2.   za cenę nie niższą niż 2.346,00 zł (dwa tysiące trzysta czterdzieści sześć złotych) netto, w przypadku gdyby aukcja przeprowadzona w terminie wskazanym w pkt 1, nie doszła do skutku ze względu na brak oferentów, jak również ustalenie, że syndyk przeprowadzi aukcję po obniżonej cenie, podaną do publicznej wiadomości, w terminie nie wcześniejszym niż po upływie dwóch tygodni od upływu terminu przeprowadzenia aukcji wskazanego w pkt 1;</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYjllNjJlNDYtMzYzMi00MTNjLWFhMTYtOTBmZGYzNzM2YmI2JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>20260407/00456</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BY1B/GUp-s/419/2025</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MAGDALENA</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>KRAJEWSKA</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Niszczewice, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>76061002002</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>5562409843</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Syndyk, którym jest Maciej Grzelak, obwieszcza, że dokumentem z dnia 31 marca 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest MAGDALENA KRAJEWSKA (PESEL 76061002002), sygnatura akt BY1B/GUp-s/419/2025
+obwieszcza:
+REGULAMIN SPRZEDAŻY Z WOLNEJ RĘKI
+W FORMIE KONKURSU OFERT
+nieruchomości w postępowaniu upadłościowym Magdaleny Krajewskiej oraz Rafała Krajewskiego osób fizycznych
+nieprowadzących działalności gospodarczej
+I. Przedmiot sprzedaży
+1. Przedmiotem sprzedaży są udziały małżonków Magdaleny i Rafała Krajewskich wynoszące po 1/2 w nieruchomości gruntowej zabudowanej budynkiem mieszkalnym, stanowiącej działkę o powierzchni 1,0100 ha o numerze 176/1, położonej w obrębie ewidencyjnym nr 0014 w Niszczewicach, dla której Sąd Rejonowy w Inowrocławiu prowadzi księgę wieczystą o numerze: BY1I/00052618/8 (numer składnika w spisie inwentarza: 2.1 Magdaleny Krajewskiej; numer składnika w spisie inwentarza: 2.1 Rafała Krajewskiego) - udziały są sprzedawane łącznie,
+2. Cena minimalna sprzedaży nieruchomości wynosi 399.000,00 zł (trzysta dziewięćdziesiąt dziewięć tysięcy złotych) – po 199.500,00 zł za każdy udział.
+3. Wpłaty wadium w wysokości 10.000,00 zł należy dokonać na rachunek bankowy masy upadłości o numerze 79 1600 1185 1779 9689 6000 0001. W tytule przelewu należy wskazać „wadium BY1B/GUp-s/419/2025”,
+4. Wadium uważa się za zapłacone jeżeli uznanie rachunku bankowego masy upadłości kwotą wadium nastąpi najpóźniej w dniu 4 maja 2026 roku.
+II. Warunki złożenia oferty i termin wyboru oferenta
+1. Przez złożenie oferty rozumie się złożenie pisemnej oferty na adres doradca restrukturyzacyjny Maciej Grzelak (ul. Gdańska 92/8, 85-021 Bydgoszcz), osobiście lub listownie w zamkniętej kopercie, która to musi wpłynąć najpóźniej do dnia 4 maja 2026 roku do godz. 13:30. W kopercie winna znajdować się kolejna zamknięta koperta zawierająca ofertę, z dopiskiem na tej kopercie „OFERTA, SYGN. AKT BY1B/GUp-s/419/2025, NIE OTWIERAĆ”.
+2. Pisemna oferta winna zawierać co najmniej:
+a) w przypadku osób fizycznych: imię i nazwisko, dokładny adres, numer telefonu oraz numer PESEL, czytelny podpis oferenta,
+w przypadku innych podmiotów niż osoba fizyczna: nazwę oferenta wraz z podaniem jego siedziby, formy organizacyjno-prawnej oraz czytelne podpisy osób upoważnionych do składania oświadczeń w imieniu oferenta wraz z dokumentem wykazującym umocowanie tych osób, dokładny adres, numer NIP lub KRS, numer telefonu,
+b) wskazanie na co składana jest oferta oraz oferowaną cenę nabycia w złotówkach, której wysokość nie może być niższa niż minimalna cena sprzedaży,
+c) w przypadku podmiotu zagranicznego zezwolenie Ministra Spraw Wewnętrznych i Administracji na zakup nieruchomości bądź oświadczenie, że zachodzą wymogi określone w art. 8 ustawy z dnia 24.03.1920 r. o nabywaniu nieruchomości przez cudzoziemców (tekst jednolity: Dz.U.2014.1380),
+d) oświadczenie oferenta, że:
+- zapoznał się z regulaminem sprzedaży, stanem prawnym i technicznym przedmiotu sprzedaży i nie wnosi do nich zastrzeżeń,
+- wyraża zgodę na wyłączenie rękojmi za wady fizyczne i prawne,
+- zobowiązuje się pokryć wszystkie koszty, podatki i opłaty związane z przeniesieniem własności nieruchomości, w tym koszty związane z zawarcie umowy sprzedaży w formie aktu notarialnego,
+- oferent zobowiązuje się dokonać zapłaty całej ceny nie później niż w dniu poprzedzającym zawarcie umowy przenoszącej prawa do nieruchomości,
+e) wszelkie zezwolenia i zgody, jeżeli ze względu na osobę nabywcy są one prawem wymagane (w tym, w przypadku nabywców niebędących osobami fizycznymi, zgodę właściwych organów nabywcy na nabycie przedmiotu sprzedaży, natomiast w przypadku braku konieczności uzyskania takiej zgody od organów nabywcy właściwe dokumenty, które to potwierdzają,
+3. Oferent może, przed upływem terminu do składania ofert, zmienić lub wycofać ofertę. W celu dokonania zmiany lub wycofania oferty, oferent złoży kolejną zapieczętowaną kopertę, oznaczoną jak opisano w punkcie II. 1 z dodaniem słowa: "Zmiana" albo "Wycofanie".
+4. Rozpoznanie złożonych ofert nastąpi w dniu 5 maja 2026 roku o godz. 9:00 w kancelarii syndyka mieszczącej się w Bydgoszczy przy ul. Gdańskiej 92/8. Podstawowe kryterium wyboru oferty stanowi najwyższa zaoferowana cena, równa co najmniej cenie wywoławczej lub wyższa od niej, z tym zastrzeżeniem, że Syndyk może:
+- dokonać swobodnego wyboru oferty albo
+- zarządzić w dniu otwarcia ofert dodatkowo aukcję (licytację) z udziałem oferentów, którzy stawili się na otwarciu ofert, na warunkach wskazanych w części III niniejszego regulaminu.
+III. Zasady przeprowadzenia aukcji (licytacji)
+1. Uczestnikami aukcji (licytacji) są oferenci, którzy stawili się w dacie otwarcia ofert w kancelarii syndyka osobiście lub przez pełnomocników.
+2. Aukcja ma formę ustną i rozpoczyna się od wywołania najwyższej ceny zaproponowanej przez oferentów w ofertach pisemnych.
+3. W trakcie aukcji oferenci zgłaszają ustnie kolejne postąpienia, nie niższe niż o 1.000,00 zł (słownie: jeden tysiąc złotych) dla nieruchomości stanowiącej przedmiot sprzedaży.
+4. Zaoferowana cena przestaje wiązać oferenta, gdy inny oferent zaoferuje wyższą cenę, a ten jej nie przebije.
+5. Syndyk wybiera ofertę uczestnika licytacji (udziela przybicia), który zaoferował najwyższą cenę, której po dwukrotnym powtórzeniu przez Syndyka nikt z uczestników nie podwyższył (trzecie powtórzenie zaoferowanej ceny jest równoznaczne z jej przyjęciem).
+6. W przypadku, gdyby żaden z oferentów nie zaoferował postąpienia tylko pozostał przy cenie wskazanej w ofercie, Syndyk dokona swobodnego wyboru oferty.
+IV. Protokół konkursu ofert i aukcji (licytacji).
+Z przebiegu Konkursu ofert i aukcji (licytacji) syndyk sporządza i podpisuje w dwóch egzemplarzach protokół, dokumentujący podstawowe czynności związane z przebiegiem Konkursu ofert, w tym:
+1. opis przedmiotu Konkursu ofert i aukcji (licytacji);
+2. imię i nazwisko lub nazwę oferentów biorących udział w Konkursie ofert i aukcji (licytacji);
+3. oferowane ceny;
+4. informację o spełnieniu przez oferentów warunków Konkursu ofert;
+5. uzasadnienie odrzucenia oferty;
+6. wskazanie wybranej oferty wraz z uzasadnieniem wyboru – w razie rozstrzygnięcia Konkursu ofert;
+7. wskazanie oferenta, któremu udzielono przybicia – w razie aukcji (licytacji);
+8. zamknięcie Konkursu ofert bez dokonania wyboru oferty
+V. Ogłoszenie wyniku konkursu ofert nastąpi niezwłocznie po jego zakończeniu.
+VI. Postanowienia ogólne
+1. Sprzedaż następuje w postępowaniu upadłościowym i stosownie do art. 313 ust. 1 Prawa upadłościowego ma skutki sprzedaży egzekucyjnej.
+2. Syndyk zastrzega sobie prawo do zmiany warunków lub odwołania procedury sprzedaży na każdym etapie bez podania przyczyny.
+3. Obowiązek zawarcia umowy sprzedaży w terminie do dnia 31 sierpnia 2026 r. pod rygorem utraty wadium.
+4. Oferent przyjmuje do wiadomości, iż na terenie nieruchomości mogą pozostawać przedmioty ruchome niestanowiące składników masy upadłości. Syndyk nie będzie zobowiązany do ich usunięcia lub uprzątnięcia.
+5. W przypadku nieruchomości zamieszkiwanej syndyk nie jest zobowiązany do zapewnienia opuszczenia i opróżnienia lokalu przez osoby dotychczas ten lokal zajmujące.
+6. Złożenie oferty jest równoznaczne z akceptacją niniejszego regulaminu oraz treści ogłoszenia.</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyZDZiOThiZjQtMzZlNy00OGE0LWIxNTItZGQ5MTg5M2U4OGMzJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>20260407/00481</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BB1B/GUp-Sędzia-upr/28/2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Danuta</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Wiercigroch</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Bielsko-Biała, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>56122111469</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Bielsku-Białej</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>VI Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy w Bielsku-Białej, VI Wydział Gospodarczy, ul. Wojciecha Bogusławskiego 24, 43-300 Bielsko-Biała, obwieszcza, że postanowieniem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Danuta Wiercigroch (PESEL 56122111469), sygnatura akt BB1B/GUp-Sędzia-upr/28/2026
+postanowił:
+1.   na zasadzie art.342a Prawa upadłościowego wydzielić upadłej kwotę 20 400 zł (dwadzieścia tysięcy czterysta złotych) z sumy uzyskanej ze sprzedaży nieruchomości tj. lokalu mieszkalnego położonego w Skoczowie przy ul. Targowej 22 nr księgi wieczystej  BB1C/00089951/6 odpowiadającej czynszowi najmu w wysokości po 1700 zł (jeden tysiąc siedemset złotych) przez okres 12 (dwunastu) miesięcy,
+2.    oddalić wniosek upadłej w pozostałym zakresie.
+Poucza się, że wierzycielowi przysługuje zażalenie na postanowienie o wyłączeniu z masy upadłości. Zażalenie wnosi się w następujący sposób: wierzyciel może w terminie tygodnia od dnia obwieszczenia postanowienia o wyłączeniu z masy upadłości, wnieść zażalenie. Zażalenie podlega opłacie w wysokości 200,00 zł. Sąd odrzuci zażalenie jeżeli będzie ono spóźnione, nieopłacone lub dotknięte brakami, które nie zostaną usunięte mimo wezwania. Zażalenie należy skierować do Sądu Upadłościowego - Sądu Rejonowego w Bielsku-Białej, VI Wydział Gospodarczy.</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyZWJhYjEzNDEtYjhiZC00ZjE0LWI2MjUtZjQ4YjMxYTA2NGI2JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>20260407/00500</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07.04.2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>WA2M/GUp-Sędzia-upr/443/2025</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Jabłonka</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Warszawa, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>87061208992</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>7822346886</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy dla m.st.Warszawy w Warszawie</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>XIX Wydział Gospodarczy</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Sąd Rejonowy dla m.st.Warszawy w Warszawie, XIX Wydział Gospodarczy, ul. Czerniakowska 100a, 00-454 Warszawa, obwieszcza, że dokumentem z dnia 7 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Adam Jabłonka (PESEL 87061208992), sygnatura akt WA2M/GUp-Sędzia-upr/443/2025
+postanowił:
+1.     wydzielić upadłemu Adamowi Jabłonka z sumy uzyskanej ze sprzedaży prawa własności nieruchomości gruntowej, stanowiącej działkę ewid. nr 105/7 obręb 0090 o pow. 0,1386 ha, zabudowaną budynkiem mieszkalnym jednorodzinnym, położoną w miejscowości Kępa Kiełpińska 12, w gminie Łomianki, w powiecie warszawskim zachodnim, w województwie mazowieckim, dla której Sąd Rejonowy dla Warszawy-Mokotowa w Warszawie X Wydział Ksiąg Wieczystych prowadzi księgę wieczystą numer WA4M/ 00396385/9, kwotę 72.000,00 zł (siedemdziesiąt dwa tysiące złotych zero groszy) na okres 24 (dwudziestu czterech) miesięcy;
+2.     oddalić wniosek w pozostałym zakresie.
+Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego dla m.st. Warszawy w Warszawie, XIX Wydział Gospodarczy. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyM2ZmYWUzZmMtMmRkZC00YjY1LThjNzMtMzQzMjRmNTk1ZjdkJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>20260406/00017</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SZ1S/GUp-s/61/2026</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Zbigniew</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Banach</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Uniemyśl, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>54032407177</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>8512599352</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Syndyk, którym jest Monika Borek, obwieszcza, że dokumentem z dnia 6 kwietnia 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest Zbigniew Banach (PESEL 54032407177), sygnatura akt SZ1S/GUp-s/61/2026
+obwieszcza:
+w trybie przepisu art. 219 ust. 1d ustawy Prawo upadłościowe, że do akt postępowania upadłościowego Zbigniewa Banacha, osoby fizycznej nieprowadzącej działalności gospodarczej, zostały złożone następujące dokumenty: spis inwentarza oraz plan likwidacyjny.</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNzFjOWJmN2YtOTE1MS00YjRhLTg2NDYtYmY2ZWRlNTA4YWE3JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>20260406/00019</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>SZ1S/GUp-s/61/2026</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Zbigniew</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Banach</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Uniemyśl, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>54032407177</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>8512599352</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Syndyk, którym jest Monika Borek, obwieszcza, że dokumentem z dnia 6 kwietnia 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest Zbigniew Banach (PESEL 54032407177), sygnatura akt SZ1S/GUp-s/61/2026
+obwieszcza:
+w trybie przepisu art. 219 ust. 1d ustawy Prawo upadłościowe, że do akt postępowania upadłościowego Zbigniewa Banacha osoby fizycznej nieprowadzącej działalności gospodarczej, został złożony następujący dokument: korekta planu likwidacyjnego.</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyOTNlMWYzOTUtMDQ5Ny00MGNjLTliNDUtMzRjNTRiNDllMTkxJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20260406/00021</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>SZ1S/GUp-s/64/2026</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Agata</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Cudzanowska</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Szczecin, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>82070118148</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
           <t>Syndyk, którym jest Monika Borek, obwieszcza, że dokumentem z dnia 6 kwietnia 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest Agata Cudzanowska (PESEL 82070118148), sygnatura akt SZ1S/GUp-s/64/2026
 obwieszcza:
 w trybie przepisu art. 219 ust. 1d ustawy Prawo upadłościowe, że do akt postępowania upadłościowego Agaty Cudzanowskiej, osoby fizycznej nieprowadzącej działalności gospodarczej, zostały złożone następujące dokumenty: spis inwentarza oraz plan likwidacyjny.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyOTYwNzc1YjMtNzQyZi00YTBlLTkxNWUtYTAwZjI5MzI5YTU3JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>20260406/00031</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>SZ1S/GUp-s/68/2026</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Agnieszka</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Musialska</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Dębina, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>67122407780</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>8521357134</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Syndyk, którym jest Monika Borek, obwieszcza, że dokumentem z dnia 6 kwietnia 2026 roku wydanym w sprawie sprawy po ogłoszeniu upadłości osób fizycznych nieprowadzących działalności gospodarczej prowadzone przez syndyka dłużnika, którym jest Agnieszka Musialska (PESEL 67122407780), sygnatura akt SZ1S/GUp-s/68/2026
+obwieszcza:
+w trybie przepisu art. 219 ust. 1d ustawy Prawo upadłościowe, że do akt postępowania upadłościowego Agnieszki Musialskiej, osoby fizycznej nieprowadzącej działalności gospodarczej, zostały złożone następujące dokumenty: spis inwentarza oraz plan likwidacyjny.</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyOTExNGMyNTYtNWM1Zi00ZmExLWEyMWEtM2I3MzU0MmRkMmVmJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>20260406/00032</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CZ1C/GUp-s/168/2024</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Krzysztof</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Grudziński</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Pawonków, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>83110518775</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>sygn. akt CZ1C/GUp-s/168/2024, znak pisma: CZ1C/GUp-s/168/2024/32
+Treść obwieszczenia syndyka
+Dnia 6 kwietnia 2026 roku
+Syndyk obwieszcza, że w postępowaniu upadłościowym dłużnika, którym jest Krzysztof Grudziński, prowadzonego pod sygn. akt: CZ1C/GUp-s/168/2024, złożono do akt opis i szacowanie:
+nieruchomości: udziału 1/2 w prawie własności do lokalu mieszkalnego o powierzchni użytkowej 92,38 m2 dla którego Sąd Rejonowy w Kluczborku, IV Wydział Ksiąg Wieczystych prowadzi księgę wieczysta nr OP1U/00057695/2
+Poucza się, że na opis i oszacowanie można wnieść zarzuty. Zarzuty wnosi się w terminie tygodnia od dnia ukazania się niniejszego obwieszczenia sędziemu-komisarzowi albo w przypadku postępowania upadłościowego prowadzonego na podstawie art. 491 (1) ust. 1 prawa upadłościowego sędziemu wyznaczonemu.
+Aby złożyć środek zaskarżenia:
+Zaloguj się do Portalu Użytkowników Zarejestrowanych,
+Na stronie głównej wybierz kafelek "Katalog dokumentów",
+W katalogu dokumentów wybierz kafelek "Środki zaskarżenia",
+Wyszukaj właściwe pismo.
+Właściwym pismem dla tego orzeczenia jest pismo o kodzie zatytułowane: "".
+Możesz również w katalogu dokumentów nacisnąć przycisk "Wyszukaj wzór pisma" i w polu wyszukiwania wpisać . W wynikach wyszukiwania należy wybrać najwyższą wersję pisma.</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMWYxMjljOTMtMDU2NC00NDgwLTk4MzktNTFlMTk1YTczMGZkJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>20260406/00033</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CZ1C/GUp-s/243/2025</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Stanisław</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Najgebauer</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Zawada, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>47050802053</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>5730037834</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>sygn. akt CZ1C/GUp-s/243/2025, znak pisma: CZ1C/GUp-s/243/2025/16
+Treść obwieszczenia syndyka
+Dnia 6 kwietnia 2026 roku
+Syndyk obwieszcza, że w postępowaniu upadłościowym dłużnika, którym jest Stanisław Najgebauer, prowadzonego pod sygn. akt: CZ1C/GUp-s/243/2025, złożono do akt opis i szacowanie:
+nieruchomości: udział w 1/2 w prawie własności do nieruchomości składającej się z działek ewidencyjnych nr 310/1, 457, 703, 310/3, 530/2, 659, 776 o łącznej pow. 3,4754 ha dla której Sąd Rejonowy w Myszkowie, V Wydział Ksiąg Wieczystych prowadzi księgę wieczysta nr CZ1M/00005710/7
+Poucza się, że na opis i oszacowanie można wnieść zarzuty. Zarzuty wnosi się w terminie tygodnia od dnia ukazania się niniejszego obwieszczenia sędziemu-komisarzowi albo w przypadku postępowania upadłościowego prowadzonego na podstawie art. 491 (1) ust. 1 prawa upadłościowego sędziemu wyznaczonemu.
+Aby złożyć środek zaskarżenia:
+Zaloguj się do Portalu Użytkowników Zarejestrowanych,
+Na stronie głównej wybierz kafelek "Katalog dokumentów",
+W katalogu dokumentów wybierz kafelek "Środki zaskarżenia",
+Wyszukaj właściwe pismo.
+Właściwym pismem dla tego orzeczenia jest pismo o kodzie zatytułowane: "".
+Możesz również w katalogu dokumentów nacisnąć przycisk "Wyszukaj wzór pisma" i w polu wyszukiwania wpisać . W wynikach wyszukiwania należy wybrać najwyższą wersję pisma.</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyODlkYjkwOTktYmEzOC00NWM2LWI0OTEtNDMxNDVlNzYxZWVkJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>20260406/00045</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BB1B/GUp-s/513/2025</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Grzegorz</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Ziemba</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Hecznarowice, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>90032314833</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>9372507846</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>sygn. akt BB1B/GUp-s/513/2025, znak pisma: BB1B/GUp-s/513/2025/27
+Treść obwieszczenia syndyka
+Dnia 6 kwietnia 2026 roku
+Syndyk obwieszcza, że w postępowaniu upadłościowym dłużnika, którym jest Grzegorz Ziemba, prowadzonego pod sygn. akt: BB1B/GUp-s/513/2025, złożono do akt opis i szacowanie udziału wynoszącego 1/8 w prawie własności nieruchomości położonej w Hecznarowicach, gmina Wilamowice, powiat bielski, dla której Sąd Rejonowy w Bielsku-Białej, VII Wydział Ksiąg Wieczystych prowadzi księgę wieczystą nr BB1B/00088834/2, składającej się z działek ewidencyjnych o numerach: 2102 o pow. 0,0972 ha zabudowanej budynkiem mieszkalnym nr 64 przy ul. Stawowej, 26/3 o pow. 0,0421 ha zabudowanej dwoma budynkami niemieszkalnymi (gospodarczymi) oraz 26/12 o pow. 0,1503 ha niezabudowanej</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMWYyZGYzNTEtMmI5OC00NjFiLTg5NTQtNWZlNGQ0NzE2ZDZjJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>20260406/00050</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>06.04.2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>LD1M/GUp-s/846/2025</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Izabela</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Jurczyk</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Łódź, Polska / POLAND</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>74070301321</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>7262141998</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>sygn. akt LD1M/GUp-s/846/2025, znak pisma: LD1M/GUp-s/846/2025/60
+Treść obwieszczenia syndyka
+Dnia 6 kwietnia 2026 roku
+Syndyk obwieszcza, że w postępowaniu upadłościowym dłużnika, którym jest Izabela Jurczyk, prowadzonego pod sygn. akt: LD1M/GUp-s/846/2025, złożono do akt opis i szacowanie:
+nieruchomości: udział 1/1 w prawie własności nieruchomości gruntowej położonej w miejscowości Wymysłów Piaski, oznaczonej zgodnie z ewidencją gruntów jako działka gruntu nr 50, obręb 0016 Wymysłów Piaski, gmina Dobroń, powiat pabianicki; nieruchomość ma powierzchnię gruntu 0,9667 ha i jest działką niezabudowana, dla której prowadzona jest księga wieczysta nr SR1L/00049949/7 przez Sąd Rejonowy w Łasku, V Wydział Ksiąg Wieczystych; dla nieruchomości wydano nieprawomocną decyzję o warunkach zabudowy 6 (sześciu) domów jednorodzinnych, decyzja została zaskarżona, jest nieprawomocna;
+Poucza się, że na opis i oszacowanie można wnieść zarzuty. Zarzuty wnosi się w terminie tygodnia od dnia ukazania się niniejszego obwieszczenia sędziemu-komisarzowi albo w przypadku postępowania upadłościowego prowadzonego na podstawie art. 491 (1) ust. 1 prawa upadłościowego sędziemu wyznaczonemu.
+Aby złożyć środek zaskarżenia:
+Zaloguj się do Portalu Użytkowników Zarejestrowanych,
+Na stronie głównej wybierz kafelek "Katalog dokumentów",
+W katalogu dokumentów wybierz kafelek "Środki zaskarżenia",
+Wyszukaj właściwe pismo.
+Właściwym pismem dla tego orzeczenia jest pismo o kodzie zatytułowane: "".
+Możesz również w katalogu dokumentów nacisnąć przycisk "Wyszukaj wzór pisma" i w polu wyszukiwania wpisać . W wynikach wyszukiwania należy wybrać najwyższą wersję pisma.</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYTU2OGJiNTktYTE5OS00YjBiLTgzYzQtZWMzZWVmMGE0MDhiJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>20260405/00001</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>05.04.2026</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>KR1S/GUp/88/2024</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Katarzyna</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Jakubowska</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Skawina, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>84020202589</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>6751275485</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 5 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza upadłego, którym jest Katarzyna Jakubowska, PESEL 84020202589, sygnatura akt KR1S/GUp/88/2024, na podstawie art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolił syndykowi na sprzedaż z wolnej ręki, po obniżonej cenie, udziału w wysokości 1/2 w prawie własności nieruchomości gruntowej położonej w przy ul. Armii Krajowej 18 w miejscowości Skawina, gm. Skawina, woj. małopolskie, obejmującej działki ewidencyjne nr 5644 i 5645, dla której Sąd Rejonowy w Wieliczce V Zamiejscowy Wydział Ksiąg Wieczystych z s. w Skawinie prowadzi księgę wieczystą nr KR3I/00008006/0 (nr 2.1 w spisie inwentarza), za najwyższą zaoferowaną cenę, nie niższą niż 250.687,50 zł (dwieście pięćdziesiąt tysięcy sześćset osiemdziesiąt siedem złotych 50/100) po przeprowadzeniu przez syndyka pisemnego konkursu ofert, o którym obwieści na co najmniej trzy tygodnie przed terminem rozstrzygnięcia konkursu na co najmniej trzech internetowych portalach branżowych.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYjRkOWFkY2YtNjVmZC00NjNkLWJhNGItNGNjOWVmOGUxYjMyJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>20260404/00007</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>04.04.2026</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>KR1S/GUp-Sędzia-upr/12/2026</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Katarzyna</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Jachyra</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Piotrowice, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>76032018700</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>5492062327</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie, VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych, ul. Przy Rondzie 7, 31-547 Kraków, obwieszcza, że postanowieniem z 4 kwietnia 2026 roku wydanym przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Katarzyna Jachyra (PESEL 76032018700), sygnatura akt KR1S/GUp-Sędzia-upr/12/2026
 obwieszcza: że w skład masy upadłości nie wchodzi wynagrodzenie upadłej Katarzyny Jachyry w całości, począwszy od miesiąca marca 2026 roku.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyMmJkYzg3ZTgtNjM0ZS00MjE3LWI2ZjUtNzRiNzhhNWNhMDhiJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>20260404/00012</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>04.04.2026</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>LU1S/GUp-Sędzia-upr/46/2026</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Łukasz</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Maciąg</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Orchówek, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
         <is>
           <t>77110706933</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>5791764391</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>Sąd Rejonowy Lublin-Wschód w Lublinie z siedzibą w Świdniku</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>IX Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 4 kwietnia 2026 roku wydanym w sprawie wnioski oraz pisma do rozpoznania przez sędziego wyznaczonego w sprawach upadłościowych osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Łukasz Maciąg , PESEL 77110706933, sygnatura akt LU1S/GUp-Sędzia-upr/46/2026, postanowił:
 I.               wyłączyć z masy upadłości Łukasza Maciąga jako osoby fizycznej nieprowadzącej działalności gospodarczej prawa majątkowe w postaci 100 udziałów w spółce LUBAVA SPÓŁKA Z OGRANICZONĄ ODPOWIEDZIALNOŚCIĄ z siedzibą w Warszawie, KRS: 0000620127, o wartości nominalnej 5000 zł (poz. 4.1 spisu inwentarza LU1S/GUp-s/232/2024/154);
@@ -885,65 +2869,65 @@
 Na niniejsze postanowienie przysługuje zażalenie do Sądu Rejonowego Lublin-Wschód w Lublinie z siedzibą w Świdniku, IX Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych. Zażalenie należy wnieść w ciągu tygodnia od dnia obwieszczenia postanowienia w Rejestrze. Zażalenie podlega opłacie w wysokości 200,00 zł.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyNjY4ODQ3ZjEtNDM1YS00NDQwLTgwNjQtY2FhMWE3NTdiNTRiJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>20260404/00018</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>04.04.2026</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>KR1S/GUp-Sędzia-upr/860/2025</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Małgorzata</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Borkowicz</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Kraków, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>72073114968</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie, VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych, ul. Przy Rondzie 7, 31-547 Kraków, obwieszcza, że postanowieniem z 4 kwietnia 2026 roku wydanym w sprawie upadłościowej osób fizycznych nieprowadzących działalności gospodarczej dłużnika, którym jest Małgorzata Borkowicz (PESEL 72073114968), sygnatura akt KR1S/GUp-Sędzia-upr/860/2025
 obwieszcza:
@@ -951,70 +2935,70 @@
 II. ustalić, że w skład masy upadłości nie wchodzą środki zgromadzone na rachunku depozytowym Domu Pomocy Społecznej przy ul. Łanowej 1B w Krakowie w kwocie 2 555,27 zł.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyZWU0YWI0ZjItNjhjMi00ZWFlLTk4YjMtYzQxYjcyNDY5ZjE5JTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>20260404/00026</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>04.04.2026</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>KR1S/GUp/98/2025</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Edyta</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Pułecka</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Spytkowice, Polska / POLAND</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Osoba fizyczna nieprowadząca działalności gospodarczej</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>76042612080</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
         <is>
           <t>Sąd Rejonowy dla Krakowa-Śródmieścia w Krakowie</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>VIII Wydział Gospodarczy dla spraw upadłościowych i restrukturyzacyjnych</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>Sędzia-komisarz obwieszcza, że postanowieniem z dnia 4 kwietnia 2026 roku wydanym w sprawie po ogłoszeniu upadłości osoby fizycznej nieprowadzącej działalności gospodarczej z udziałem sędziego-komisarza upadłego, którym jest Edyta Pułecka , PESEL 76042612080, sygnatura akt KR1S/GUp/98/2025, postanowił podstawie art. 206 ust. 1 pkt 3 w zw. z art. 213 ust. 1 ustawy z dnia 28 lutego 2003r. Prawo upadłościowe zezwolić syndykowi na sprzedaż z wolnej ręki, mienia wchodzącego w skład masy upadłości w postaci udziału w wysokości 1/2 części w prawie własności nieruchomości gruntowej zabudowanej, składającej się z działki ewidencyjnej nr 4883/34, o powierzchni 0,0655 ha, położonej w Spytkowicach, woj. małopolskie, objętej księgą wieczystą numer KR1W/00039427/1, za najwyższą zaoferowaną cenę, nie niższą niż wartość oszacowania tj. za kwotę nie niższą niż 318.000,00 zł (trzysta osiemnaście tysięcy złotych 00/100), po przeprowadzeniu przez syndyka pisemnego konkursu ofert, o którym obwieści na co najmniej dwa tygodnie przed terminem rozstrzygnięcia konkursu w prasie o zasięgu lokalnym oraz na co najmniej dwóch internetowych portalach branżowych.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>https://krz.ms.gov.pl/#!/application/KRZPortalPUB/1.9/KrzRejPubGui.SzczegolyObwieszczenia?params=JTdCJTIyaWRaZXduZXRyem55JTIyJTNBJTIyYjU3MWM5NzItYzE3Ni00Yzc2LTliNWItODJkZDFhMzBiMmYzJTIyJTJDJTIydWtyeWpXc3RlY3olMjIlM0F0cnVlJTdE</t>
         </is>
@@ -1030,6 +3014,35 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>